<commit_message>
ders kararları bölümü güncelenmesi
</commit_message>
<xml_diff>
--- a/data/kriter_veri_seti_2022.xlsx
+++ b/data/kriter_veri_seti_2022.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,26 @@
           <t>kayitli_ogrenci</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>katilim_sayisi</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>toplam_hafta</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>katilim_yuzdesi</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>devamsiz_ogrenci_sayisi</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -517,6 +537,18 @@
       <c r="K2" t="n">
         <v>50</v>
       </c>
+      <c r="L2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="M2" t="n">
+        <v>14</v>
+      </c>
+      <c r="N2" t="n">
+        <v>85.59</v>
+      </c>
+      <c r="O2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -562,6 +594,18 @@
       <c r="K3" t="n">
         <v>50</v>
       </c>
+      <c r="L3" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="M3" t="n">
+        <v>14</v>
+      </c>
+      <c r="N3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -607,6 +651,18 @@
       <c r="K4" t="n">
         <v>50</v>
       </c>
+      <c r="L4" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="M4" t="n">
+        <v>14</v>
+      </c>
+      <c r="N4" t="n">
+        <v>84.01000000000001</v>
+      </c>
+      <c r="O4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -652,6 +708,18 @@
       <c r="K5" t="n">
         <v>50</v>
       </c>
+      <c r="L5" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>14</v>
+      </c>
+      <c r="N5" t="n">
+        <v>86.44</v>
+      </c>
+      <c r="O5" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -697,6 +765,18 @@
       <c r="K6" t="n">
         <v>50</v>
       </c>
+      <c r="L6" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="M6" t="n">
+        <v>14</v>
+      </c>
+      <c r="N6" t="n">
+        <v>84.29000000000001</v>
+      </c>
+      <c r="O6" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -742,6 +822,18 @@
       <c r="K7" t="n">
         <v>50</v>
       </c>
+      <c r="L7" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="M7" t="n">
+        <v>14</v>
+      </c>
+      <c r="N7" t="n">
+        <v>87.01000000000001</v>
+      </c>
+      <c r="O7" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -787,6 +879,18 @@
       <c r="K8" t="n">
         <v>50</v>
       </c>
+      <c r="L8" t="n">
+        <v>12.02</v>
+      </c>
+      <c r="M8" t="n">
+        <v>14</v>
+      </c>
+      <c r="N8" t="n">
+        <v>85.87</v>
+      </c>
+      <c r="O8" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -832,6 +936,18 @@
       <c r="K9" t="n">
         <v>50</v>
       </c>
+      <c r="L9" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="M9" t="n">
+        <v>14</v>
+      </c>
+      <c r="N9" t="n">
+        <v>88.01000000000001</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -877,6 +993,18 @@
       <c r="K10" t="n">
         <v>50</v>
       </c>
+      <c r="L10" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="M10" t="n">
+        <v>14</v>
+      </c>
+      <c r="N10" t="n">
+        <v>82.72</v>
+      </c>
+      <c r="O10" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -922,6 +1050,18 @@
       <c r="K11" t="n">
         <v>50</v>
       </c>
+      <c r="L11" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="M11" t="n">
+        <v>14</v>
+      </c>
+      <c r="N11" t="n">
+        <v>83.29000000000001</v>
+      </c>
+      <c r="O11" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -967,6 +1107,18 @@
       <c r="K12" t="n">
         <v>50</v>
       </c>
+      <c r="L12" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="M12" t="n">
+        <v>14</v>
+      </c>
+      <c r="N12" t="n">
+        <v>82.86</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1012,6 +1164,18 @@
       <c r="K13" t="n">
         <v>50</v>
       </c>
+      <c r="L13" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="M13" t="n">
+        <v>14</v>
+      </c>
+      <c r="N13" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="O13" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1057,6 +1221,18 @@
       <c r="K14" t="n">
         <v>50</v>
       </c>
+      <c r="L14" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="M14" t="n">
+        <v>14</v>
+      </c>
+      <c r="N14" t="n">
+        <v>85.15000000000001</v>
+      </c>
+      <c r="O14" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1102,6 +1278,18 @@
       <c r="K15" t="n">
         <v>50</v>
       </c>
+      <c r="L15" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="M15" t="n">
+        <v>14</v>
+      </c>
+      <c r="N15" t="n">
+        <v>83.58</v>
+      </c>
+      <c r="O15" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1147,6 +1335,18 @@
       <c r="K16" t="n">
         <v>50</v>
       </c>
+      <c r="L16" t="n">
+        <v>12.26</v>
+      </c>
+      <c r="M16" t="n">
+        <v>14</v>
+      </c>
+      <c r="N16" t="n">
+        <v>87.58</v>
+      </c>
+      <c r="O16" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1192,6 +1392,18 @@
       <c r="K17" t="n">
         <v>50</v>
       </c>
+      <c r="L17" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="M17" t="n">
+        <v>14</v>
+      </c>
+      <c r="N17" t="n">
+        <v>85.01000000000001</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1237,6 +1449,18 @@
       <c r="K18" t="n">
         <v>50</v>
       </c>
+      <c r="L18" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="M18" t="n">
+        <v>14</v>
+      </c>
+      <c r="N18" t="n">
+        <v>84.44</v>
+      </c>
+      <c r="O18" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1282,6 +1506,18 @@
       <c r="K19" t="n">
         <v>50</v>
       </c>
+      <c r="L19" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="M19" t="n">
+        <v>14</v>
+      </c>
+      <c r="N19" t="n">
+        <v>84.58</v>
+      </c>
+      <c r="O19" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1327,6 +1563,18 @@
       <c r="K20" t="n">
         <v>50</v>
       </c>
+      <c r="L20" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="M20" t="n">
+        <v>14</v>
+      </c>
+      <c r="N20" t="n">
+        <v>86.01000000000001</v>
+      </c>
+      <c r="O20" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1372,6 +1620,18 @@
       <c r="K21" t="n">
         <v>50</v>
       </c>
+      <c r="L21" t="n">
+        <v>12.14</v>
+      </c>
+      <c r="M21" t="n">
+        <v>14</v>
+      </c>
+      <c r="N21" t="n">
+        <v>86.72</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1417,6 +1677,18 @@
       <c r="K22" t="n">
         <v>50</v>
       </c>
+      <c r="L22" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="M22" t="n">
+        <v>14</v>
+      </c>
+      <c r="N22" t="n">
+        <v>84.43000000000001</v>
+      </c>
+      <c r="O22" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1462,6 +1734,18 @@
       <c r="K23" t="n">
         <v>50</v>
       </c>
+      <c r="L23" t="n">
+        <v>12.52</v>
+      </c>
+      <c r="M23" t="n">
+        <v>14</v>
+      </c>
+      <c r="N23" t="n">
+        <v>89.43000000000001</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1507,6 +1791,18 @@
       <c r="K24" t="n">
         <v>50</v>
       </c>
+      <c r="L24" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="M24" t="n">
+        <v>14</v>
+      </c>
+      <c r="N24" t="n">
+        <v>85.15000000000001</v>
+      </c>
+      <c r="O24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1552,6 +1848,18 @@
       <c r="K25" t="n">
         <v>50</v>
       </c>
+      <c r="L25" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="M25" t="n">
+        <v>14</v>
+      </c>
+      <c r="N25" t="n">
+        <v>88.87</v>
+      </c>
+      <c r="O25" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1597,6 +1905,18 @@
       <c r="K26" t="n">
         <v>50</v>
       </c>
+      <c r="L26" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="M26" t="n">
+        <v>14</v>
+      </c>
+      <c r="N26" t="n">
+        <v>84.16</v>
+      </c>
+      <c r="O26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1642,6 +1962,18 @@
       <c r="K27" t="n">
         <v>50</v>
       </c>
+      <c r="L27" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="M27" t="n">
+        <v>14</v>
+      </c>
+      <c r="N27" t="n">
+        <v>87.29000000000001</v>
+      </c>
+      <c r="O27" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1687,6 +2019,18 @@
       <c r="K28" t="n">
         <v>50</v>
       </c>
+      <c r="L28" t="n">
+        <v>11.74</v>
+      </c>
+      <c r="M28" t="n">
+        <v>14</v>
+      </c>
+      <c r="N28" t="n">
+        <v>83.86</v>
+      </c>
+      <c r="O28" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1732,6 +2076,18 @@
       <c r="K29" t="n">
         <v>50</v>
       </c>
+      <c r="L29" t="n">
+        <v>12.12</v>
+      </c>
+      <c r="M29" t="n">
+        <v>14</v>
+      </c>
+      <c r="N29" t="n">
+        <v>86.58</v>
+      </c>
+      <c r="O29" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1777,6 +2133,18 @@
       <c r="K30" t="n">
         <v>50</v>
       </c>
+      <c r="L30" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="M30" t="n">
+        <v>14</v>
+      </c>
+      <c r="N30" t="n">
+        <v>85.15000000000001</v>
+      </c>
+      <c r="O30" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1822,6 +2190,18 @@
       <c r="K31" t="n">
         <v>50</v>
       </c>
+      <c r="L31" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="M31" t="n">
+        <v>14</v>
+      </c>
+      <c r="N31" t="n">
+        <v>85.01000000000001</v>
+      </c>
+      <c r="O31" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1867,6 +2247,18 @@
       <c r="K32" t="n">
         <v>50</v>
       </c>
+      <c r="L32" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="M32" t="n">
+        <v>14</v>
+      </c>
+      <c r="N32" t="n">
+        <v>84.56999999999999</v>
+      </c>
+      <c r="O32" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1912,6 +2304,18 @@
       <c r="K33" t="n">
         <v>50</v>
       </c>
+      <c r="L33" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="M33" t="n">
+        <v>14</v>
+      </c>
+      <c r="N33" t="n">
+        <v>84.86</v>
+      </c>
+      <c r="O33" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1957,6 +2361,18 @@
       <c r="K34" t="n">
         <v>50</v>
       </c>
+      <c r="L34" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="M34" t="n">
+        <v>14</v>
+      </c>
+      <c r="N34" t="n">
+        <v>81.29000000000001</v>
+      </c>
+      <c r="O34" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2002,6 +2418,18 @@
       <c r="K35" t="n">
         <v>50</v>
       </c>
+      <c r="L35" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="M35" t="n">
+        <v>14</v>
+      </c>
+      <c r="N35" t="n">
+        <v>85.01000000000001</v>
+      </c>
+      <c r="O35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2047,6 +2475,18 @@
       <c r="K36" t="n">
         <v>50</v>
       </c>
+      <c r="L36" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="M36" t="n">
+        <v>14</v>
+      </c>
+      <c r="N36" t="n">
+        <v>85.44</v>
+      </c>
+      <c r="O36" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2092,6 +2532,18 @@
       <c r="K37" t="n">
         <v>50</v>
       </c>
+      <c r="L37" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="M37" t="n">
+        <v>14</v>
+      </c>
+      <c r="N37" t="n">
+        <v>84.01000000000001</v>
+      </c>
+      <c r="O37" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2137,6 +2589,18 @@
       <c r="K38" t="n">
         <v>50</v>
       </c>
+      <c r="L38" t="n">
+        <v>11.74</v>
+      </c>
+      <c r="M38" t="n">
+        <v>14</v>
+      </c>
+      <c r="N38" t="n">
+        <v>83.86</v>
+      </c>
+      <c r="O38" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2182,6 +2646,18 @@
       <c r="K39" t="n">
         <v>50</v>
       </c>
+      <c r="L39" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="M39" t="n">
+        <v>14</v>
+      </c>
+      <c r="N39" t="n">
+        <v>85.15000000000001</v>
+      </c>
+      <c r="O39" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2227,6 +2703,18 @@
       <c r="K40" t="n">
         <v>50</v>
       </c>
+      <c r="L40" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="M40" t="n">
+        <v>14</v>
+      </c>
+      <c r="N40" t="n">
+        <v>85.44</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2272,6 +2760,18 @@
       <c r="K41" t="n">
         <v>50</v>
       </c>
+      <c r="L41" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="M41" t="n">
+        <v>14</v>
+      </c>
+      <c r="N41" t="n">
+        <v>88.01000000000001</v>
+      </c>
+      <c r="O41" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2317,6 +2817,18 @@
       <c r="K42" t="n">
         <v>50</v>
       </c>
+      <c r="L42" t="n">
+        <v>11.46</v>
+      </c>
+      <c r="M42" t="n">
+        <v>14</v>
+      </c>
+      <c r="N42" t="n">
+        <v>81.86</v>
+      </c>
+      <c r="O42" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2362,6 +2874,18 @@
       <c r="K43" t="n">
         <v>50</v>
       </c>
+      <c r="L43" t="n">
+        <v>11.72</v>
+      </c>
+      <c r="M43" t="n">
+        <v>14</v>
+      </c>
+      <c r="N43" t="n">
+        <v>83.72</v>
+      </c>
+      <c r="O43" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2407,6 +2931,18 @@
       <c r="K44" t="n">
         <v>50</v>
       </c>
+      <c r="L44" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="M44" t="n">
+        <v>14</v>
+      </c>
+      <c r="N44" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="O44" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2452,6 +2988,18 @@
       <c r="K45" t="n">
         <v>50</v>
       </c>
+      <c r="L45" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="M45" t="n">
+        <v>14</v>
+      </c>
+      <c r="N45" t="n">
+        <v>82.58</v>
+      </c>
+      <c r="O45" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2497,6 +3045,18 @@
       <c r="K46" t="n">
         <v>50</v>
       </c>
+      <c r="L46" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="M46" t="n">
+        <v>14</v>
+      </c>
+      <c r="N46" t="n">
+        <v>83.01000000000001</v>
+      </c>
+      <c r="O46" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2542,6 +3102,18 @@
       <c r="K47" t="n">
         <v>50</v>
       </c>
+      <c r="L47" t="n">
+        <v>11.48</v>
+      </c>
+      <c r="M47" t="n">
+        <v>14</v>
+      </c>
+      <c r="N47" t="n">
+        <v>82</v>
+      </c>
+      <c r="O47" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2587,6 +3159,18 @@
       <c r="K48" t="n">
         <v>50</v>
       </c>
+      <c r="L48" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="M48" t="n">
+        <v>14</v>
+      </c>
+      <c r="N48" t="n">
+        <v>84.87</v>
+      </c>
+      <c r="O48" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2632,6 +3216,18 @@
       <c r="K49" t="n">
         <v>50</v>
       </c>
+      <c r="L49" t="n">
+        <v>11.72</v>
+      </c>
+      <c r="M49" t="n">
+        <v>14</v>
+      </c>
+      <c r="N49" t="n">
+        <v>83.73</v>
+      </c>
+      <c r="O49" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2677,6 +3273,18 @@
       <c r="K50" t="n">
         <v>50</v>
       </c>
+      <c r="L50" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="M50" t="n">
+        <v>14</v>
+      </c>
+      <c r="N50" t="n">
+        <v>84.15000000000001</v>
+      </c>
+      <c r="O50" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2722,6 +3330,18 @@
       <c r="K51" t="n">
         <v>50</v>
       </c>
+      <c r="L51" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="M51" t="n">
+        <v>14</v>
+      </c>
+      <c r="N51" t="n">
+        <v>86.01000000000001</v>
+      </c>
+      <c r="O51" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2767,6 +3387,18 @@
       <c r="K52" t="n">
         <v>50</v>
       </c>
+      <c r="L52" t="n">
+        <v>12.14</v>
+      </c>
+      <c r="M52" t="n">
+        <v>14</v>
+      </c>
+      <c r="N52" t="n">
+        <v>86.72</v>
+      </c>
+      <c r="O52" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2812,6 +3444,18 @@
       <c r="K53" t="n">
         <v>50</v>
       </c>
+      <c r="L53" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="M53" t="n">
+        <v>14</v>
+      </c>
+      <c r="N53" t="n">
+        <v>83.29000000000001</v>
+      </c>
+      <c r="O53" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2857,6 +3501,18 @@
       <c r="K54" t="n">
         <v>50</v>
       </c>
+      <c r="L54" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="M54" t="n">
+        <v>14</v>
+      </c>
+      <c r="N54" t="n">
+        <v>79.70999999999999</v>
+      </c>
+      <c r="O54" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2902,6 +3558,18 @@
       <c r="K55" t="n">
         <v>50</v>
       </c>
+      <c r="L55" t="n">
+        <v>11.72</v>
+      </c>
+      <c r="M55" t="n">
+        <v>14</v>
+      </c>
+      <c r="N55" t="n">
+        <v>83.73</v>
+      </c>
+      <c r="O55" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2947,6 +3615,18 @@
       <c r="K56" t="n">
         <v>50</v>
       </c>
+      <c r="L56" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="M56" t="n">
+        <v>14</v>
+      </c>
+      <c r="N56" t="n">
+        <v>83.01000000000001</v>
+      </c>
+      <c r="O56" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2992,6 +3672,18 @@
       <c r="K57" t="n">
         <v>50</v>
       </c>
+      <c r="L57" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="M57" t="n">
+        <v>14</v>
+      </c>
+      <c r="N57" t="n">
+        <v>82.29000000000001</v>
+      </c>
+      <c r="O57" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3037,6 +3729,18 @@
       <c r="K58" t="n">
         <v>50</v>
       </c>
+      <c r="L58" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="M58" t="n">
+        <v>14</v>
+      </c>
+      <c r="N58" t="n">
+        <v>77.15000000000001</v>
+      </c>
+      <c r="O58" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3082,6 +3786,18 @@
       <c r="K59" t="n">
         <v>50</v>
       </c>
+      <c r="L59" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="M59" t="n">
+        <v>14</v>
+      </c>
+      <c r="N59" t="n">
+        <v>78.72</v>
+      </c>
+      <c r="O59" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3127,6 +3843,18 @@
       <c r="K60" t="n">
         <v>50</v>
       </c>
+      <c r="L60" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="M60" t="n">
+        <v>14</v>
+      </c>
+      <c r="N60" t="n">
+        <v>76.58</v>
+      </c>
+      <c r="O60" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3172,6 +3900,18 @@
       <c r="K61" t="n">
         <v>50</v>
       </c>
+      <c r="L61" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="M61" t="n">
+        <v>14</v>
+      </c>
+      <c r="N61" t="n">
+        <v>77</v>
+      </c>
+      <c r="O61" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3217,6 +3957,18 @@
       <c r="K62" t="n">
         <v>50</v>
       </c>
+      <c r="L62" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="M62" t="n">
+        <v>14</v>
+      </c>
+      <c r="N62" t="n">
+        <v>80.58</v>
+      </c>
+      <c r="O62" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3262,6 +4014,18 @@
       <c r="K63" t="n">
         <v>50</v>
       </c>
+      <c r="L63" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M63" t="n">
+        <v>14</v>
+      </c>
+      <c r="N63" t="n">
+        <v>81.15000000000001</v>
+      </c>
+      <c r="O63" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3307,6 +4071,18 @@
       <c r="K64" t="n">
         <v>50</v>
       </c>
+      <c r="L64" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="M64" t="n">
+        <v>14</v>
+      </c>
+      <c r="N64" t="n">
+        <v>78.72</v>
+      </c>
+      <c r="O64" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3352,6 +4128,18 @@
       <c r="K65" t="n">
         <v>50</v>
       </c>
+      <c r="L65" t="n">
+        <v>11</v>
+      </c>
+      <c r="M65" t="n">
+        <v>14</v>
+      </c>
+      <c r="N65" t="n">
+        <v>78.58</v>
+      </c>
+      <c r="O65" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3397,6 +4185,18 @@
       <c r="K66" t="n">
         <v>50</v>
       </c>
+      <c r="L66" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="M66" t="n">
+        <v>14</v>
+      </c>
+      <c r="N66" t="n">
+        <v>80.29000000000001</v>
+      </c>
+      <c r="O66" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3442,6 +4242,18 @@
       <c r="K67" t="n">
         <v>50</v>
       </c>
+      <c r="L67" t="n">
+        <v>11.12</v>
+      </c>
+      <c r="M67" t="n">
+        <v>14</v>
+      </c>
+      <c r="N67" t="n">
+        <v>79.43000000000001</v>
+      </c>
+      <c r="O67" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3487,6 +4299,18 @@
       <c r="K68" t="n">
         <v>50</v>
       </c>
+      <c r="L68" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="M68" t="n">
+        <v>14</v>
+      </c>
+      <c r="N68" t="n">
+        <v>80.43000000000001</v>
+      </c>
+      <c r="O68" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3532,6 +4356,18 @@
       <c r="K69" t="n">
         <v>50</v>
       </c>
+      <c r="L69" t="n">
+        <v>11.14</v>
+      </c>
+      <c r="M69" t="n">
+        <v>14</v>
+      </c>
+      <c r="N69" t="n">
+        <v>79.58</v>
+      </c>
+      <c r="O69" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3577,6 +4413,18 @@
       <c r="K70" t="n">
         <v>50</v>
       </c>
+      <c r="L70" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="M70" t="n">
+        <v>14</v>
+      </c>
+      <c r="N70" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="O70" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3622,6 +4470,18 @@
       <c r="K71" t="n">
         <v>50</v>
       </c>
+      <c r="L71" t="n">
+        <v>11.42</v>
+      </c>
+      <c r="M71" t="n">
+        <v>14</v>
+      </c>
+      <c r="N71" t="n">
+        <v>81.56999999999999</v>
+      </c>
+      <c r="O71" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3667,6 +4527,18 @@
       <c r="K72" t="n">
         <v>50</v>
       </c>
+      <c r="L72" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="M72" t="n">
+        <v>14</v>
+      </c>
+      <c r="N72" t="n">
+        <v>84.15000000000001</v>
+      </c>
+      <c r="O72" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3711,6 +4583,18 @@
       </c>
       <c r="K73" t="n">
         <v>50</v>
+      </c>
+      <c r="L73" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="M73" t="n">
+        <v>14</v>
+      </c>
+      <c r="N73" t="n">
+        <v>79.70999999999999</v>
+      </c>
+      <c r="O73" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>